<commit_message>
release: restore the delimited exports at 2.1.0
The previous commit replaced the enrichment workbooks but dropped their
zipped CSV and TSV siblings, which carry the same Provenance sheet and so
also had to be regenerated. All three formats are back for both
directions, and the GO annotation workbook is refreshed alongside them.
</commit_message>
<xml_diff>
--- a/example_analysis/4_go_enrichment/down-regulated_306/results/orthogather_GOenrichment-results_fg306_evidence-all_2026-09-14.xlsx
+++ b/example_analysis/4_go_enrichment/down-regulated_306/results/orthogather_GOenrichment-results_fg306_evidence-all_2026-09-14.xlsx
@@ -298,7 +298,7 @@
     <t>2.1.0</t>
   </si>
   <si>
-    <t>2026-09-13T23:00:14.803866+00:00</t>
+    <t>2026-09-13T23:03:10.876558+00:00</t>
   </si>
   <si>
     <t>UniProt (rest.uniprot.org)</t>
@@ -328,7 +328,7 @@
     <t>http://purl.obolibrary.org/obo/go/releases/2026-07-26/extensions/go-plus.ofn</t>
   </si>
   <si>
-    <t>2026-09-13T22:59:52.530909+00:00</t>
+    <t>2026-09-13T23:02:49.348340+00:00</t>
   </si>
   <si>
     <t>EBI GOA proteomes (ftp.ebi.ac.uk/pub/databases/GO/goa/proteomes)</t>

</xml_diff>